<commit_message>
dashboard: replace meta-refresh with JS polling via /dashboard/data JSON endpoint
</commit_message>
<xml_diff>
--- a/sub-programs.xlsx
+++ b/sub-programs.xlsx
@@ -29,9 +29,8 @@
       <text>
         <r>
           <rPr>
-            <sz val="11"/>
-            <color rgb="FF000000"/>
-            <rFont val="Calibri"/>
+            <sz val="10"/>
+            <rFont val="Arial"/>
             <family val="2"/>
             <charset val="1"/>
           </rPr>
@@ -83,9 +82,8 @@
       <text>
         <r>
           <rPr>
-            <sz val="11"/>
-            <color rgb="FF000000"/>
-            <rFont val="Calibri"/>
+            <sz val="10"/>
+            <rFont val="Arial"/>
             <family val="2"/>
             <charset val="1"/>
           </rPr>
@@ -120,7 +118,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="63">
   <si>
     <t xml:space="preserve">Programs</t>
   </si>
@@ -183,6 +181,9 @@
   </si>
   <si>
     <t xml:space="preserve">ministries to follow up each meeting</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sunday Service Plan</t>
   </si>
   <si>
     <t xml:space="preserve">Plan for next Sunday</t>
@@ -316,11 +317,12 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="m/d/yyyy"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="10">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -369,13 +371,6 @@
     </font>
     <font>
       <b val="true"/>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -554,7 +549,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D52"/>
-  <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.55078125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="19.35"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="11.85"/>
@@ -704,13 +699,13 @@
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>4</v>
+        <v>21</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>7</v>
@@ -722,7 +717,7 @@
         <v>8</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D14" s="1"/>
     </row>
@@ -732,7 +727,7 @@
         <v>8</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D15" s="1"/>
     </row>
@@ -742,7 +737,7 @@
         <v>8</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D16" s="1"/>
     </row>
@@ -752,7 +747,7 @@
         <v>8</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D17" s="1"/>
     </row>
@@ -762,7 +757,7 @@
         <v>8</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D18" s="1"/>
     </row>
@@ -772,7 +767,7 @@
         <v>8</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D19" s="1"/>
     </row>
@@ -782,7 +777,7 @@
         <v>8</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D20" s="1"/>
     </row>
@@ -792,7 +787,7 @@
         <v>8</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D21" s="1"/>
     </row>
@@ -802,7 +797,7 @@
         <v>8</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D22" s="1"/>
     </row>
@@ -812,7 +807,7 @@
         <v>8</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D23" s="1"/>
     </row>
@@ -822,7 +817,7 @@
         <v>8</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D24" s="1"/>
     </row>
@@ -832,7 +827,7 @@
         <v>8</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D25" s="1"/>
     </row>
@@ -842,7 +837,7 @@
         <v>8</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D26" s="1"/>
     </row>
@@ -852,7 +847,7 @@
         <v>8</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D27" s="1"/>
     </row>
@@ -862,7 +857,7 @@
         <v>8</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D28" s="1"/>
     </row>
@@ -872,7 +867,7 @@
         <v>8</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D29" s="1"/>
     </row>
@@ -882,7 +877,7 @@
         <v>8</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="D30" s="1"/>
     </row>
@@ -892,7 +887,7 @@
         <v>8</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D31" s="1"/>
     </row>
@@ -902,7 +897,7 @@
         <v>8</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D32" s="1"/>
     </row>
@@ -912,31 +907,31 @@
         <v>8</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D33" s="1"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B34" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D34" s="1"/>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D35" s="1"/>
     </row>
@@ -946,7 +941,7 @@
         <v>8</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D36" s="1"/>
     </row>
@@ -956,7 +951,7 @@
         <v>8</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D37" s="1"/>
     </row>
@@ -966,19 +961,19 @@
         <v>8</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D38" s="1"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B39" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D39" s="1"/>
     </row>
@@ -988,7 +983,7 @@
         <v>8</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D40" s="1"/>
     </row>
@@ -998,7 +993,7 @@
         <v>8</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D41" s="1"/>
     </row>
@@ -1008,7 +1003,7 @@
         <v>8</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D42" s="1"/>
     </row>
@@ -1018,7 +1013,7 @@
         <v>8</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D43" s="1"/>
     </row>
@@ -1028,103 +1023,103 @@
         <v>8</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D44" s="1"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B45" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D45" s="1"/>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B46" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D46" s="1"/>
     </row>
     <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B47" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="D47" s="1"/>
     </row>
     <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B48" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C48" s="8" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D48" s="1"/>
     </row>
     <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B49" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C49" s="8" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D49" s="1"/>
     </row>
     <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B50" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C50" s="8" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D50" s="1"/>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B51" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C51" s="8" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D51" s="1"/>
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="1" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B52" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C52" s="8" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="D52" s="1"/>
     </row>

</xml_diff>